<commit_message>
Feat : Fixing Bug on Download Penyelesaian
</commit_message>
<xml_diff>
--- a/Assets/harta-gonogini-transactions-20260510.xlsx
+++ b/Assets/harta-gonogini-transactions-20260510.xlsx
@@ -5,21 +5,23 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mohammad Haqqi\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Haqqi\Proyek Mini\Harta Gono Gini\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7020"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7020" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="harta-gonogini-transactions-202" sheetId="1" r:id="rId1"/>
+    <sheet name="harta-gonogini-transactions (2)" sheetId="2" r:id="rId2"/>
+    <sheet name="raw data" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="24">
   <si>
     <t xml:space="preserve">							</t>
   </si>
@@ -51,9 +53,6 @@
     <t>Astro</t>
   </si>
   <si>
-    <t>lainnya</t>
-  </si>
-  <si>
     <t>Haqqi</t>
   </si>
   <si>
@@ -61,6 +60,39 @@
   </si>
   <si>
     <t>Pending</t>
+  </si>
+  <si>
+    <t>Lintang</t>
+  </si>
+  <si>
+    <t>belanja</t>
+  </si>
+  <si>
+    <t>Sayur</t>
+  </si>
+  <si>
+    <t>Qulub(11200)(Sayur); Yohn(11200)(Sayur); Lintang(11200)(Sayur); Aldo(11200)(Sayur); Haqqi(11200)(Sayur); Acha(11200)(Sayur)</t>
+  </si>
+  <si>
+    <t>Qulub</t>
+  </si>
+  <si>
+    <t>Yohn</t>
+  </si>
+  <si>
+    <t>Aldo</t>
+  </si>
+  <si>
+    <t>Uduksss</t>
+  </si>
+  <si>
+    <t>Karaokee</t>
+  </si>
+  <si>
+    <t>Acha</t>
+  </si>
+  <si>
+    <t>Selesai</t>
   </si>
 </sst>
 </file>
@@ -203,7 +235,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -381,6 +413,18 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -544,9 +588,20 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -873,6 +928,7 @@
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
     <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -901,7 +957,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -912,24 +968,45 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
         <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
       </c>
       <c r="F2">
         <v>273000</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
         <v>12</v>
       </c>
-      <c r="H2" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>0</v>
+      <c r="F3">
+        <v>67000</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -965,4 +1042,585 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.85546875" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2">
+        <f>SUM(J2:O2)</f>
+        <v>150000</v>
+      </c>
+      <c r="G2" s="2" t="str">
+        <f>IF(OR(J2="",J2=0,J2="-"),"",J$1&amp;"("&amp;J2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(K2="",K2=0,K2="-"),"",IF(J2="", "", "; ")&amp;K$1&amp;"("&amp;K2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(L2="",L2=0,L2="-"),"", "; "&amp;L$1&amp;"("&amp;L2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(M2="",M2=0,M2="-"),"", "; "&amp;M$1&amp;"("&amp;M2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(N2="",N2=0,N2="-"),"", "; "&amp;N$1&amp;"("&amp;N2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(O2="",O2=0,O2="-"),"", "; "&amp;O$1&amp;"("&amp;O2&amp;")("&amp;$C2&amp;")")</f>
+        <v>Qulub(25000)(Astro); Lintang(25000)(Astro); Yohn(25000)(Astro); Aldo(25000)(Astro); Haqqi(25000)(Astro); Acha(25000)(Astro)</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2">
+        <f>100000/4</f>
+        <v>25000</v>
+      </c>
+      <c r="K2">
+        <f t="shared" ref="K2:O2" si="0">100000/4</f>
+        <v>25000</v>
+      </c>
+      <c r="L2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="M2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="N2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="O2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3">
+        <v>273000</v>
+      </c>
+      <c r="G3" s="2" t="str">
+        <f>IF(OR(J3="",J3=0,J3="-"),"",J$1&amp;"("&amp;J3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(K3="",K3=0,K3="-"),"",IF(J3="", "", "; ")&amp;K$1&amp;"("&amp;K3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(L3="",L3=0,L3="-"),"", "; "&amp;L$1&amp;"("&amp;L3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(M3="",M3=0,M3="-"),"", "; "&amp;M$1&amp;"("&amp;M3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(N3="",N3=0,N3="-"),"", "; "&amp;N$1&amp;"("&amp;N3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(O3="",O3=0,O3="-"),"", "; "&amp;O$1&amp;"("&amp;O3&amp;")("&amp;$C3&amp;")")</f>
+        <v>Qulub(45000)(Uduksss); Lintang(23000)(Uduksss); Yohn(45000)(Uduksss); Aldo(43000)(Uduksss); Acha(34200)(Uduksss)</v>
+      </c>
+      <c r="H3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>45000</v>
+      </c>
+      <c r="K3">
+        <v>23000</v>
+      </c>
+      <c r="L3">
+        <v>45000</v>
+      </c>
+      <c r="M3">
+        <v>43000</v>
+      </c>
+      <c r="O3">
+        <v>34200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1">
+        <v>46270</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4">
+        <v>273000</v>
+      </c>
+      <c r="G4" s="2" t="str">
+        <f t="shared" ref="G4:G10" si="1">IF(OR(J4="",J4=0,J4="-"),"",J$1&amp;"("&amp;J4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(K4="",K4=0,K4="-"),"",IF(J4="", "", "; ")&amp;K$1&amp;"("&amp;K4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(L4="",L4=0,L4="-"),"", "; "&amp;L$1&amp;"("&amp;L4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(M4="",M4=0,M4="-"),"", "; "&amp;M$1&amp;"("&amp;M4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(N4="",N4=0,N4="-"),"", "; "&amp;N$1&amp;"("&amp;N4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(O4="",O4=0,O4="-"),"", "; "&amp;O$1&amp;"("&amp;O4&amp;")("&amp;$C4&amp;")")</f>
+        <v>Qulub(45000)(Karaokee); Lintang(23000)(Karaokee); Acha(34200)(Karaokee)</v>
+      </c>
+      <c r="H4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4">
+        <v>45000</v>
+      </c>
+      <c r="K4">
+        <v>23000</v>
+      </c>
+      <c r="O4">
+        <v>34200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="G10" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="48.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>46270</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <f>SUM(I2:N2)</f>
+        <v>150000</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <f>IF(OR(I2="",I2=0,I2="-"),"",I$1&amp;"("&amp;I2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(J2="",J2=0,J2="-"),"",IF(I2="", "", "; ")&amp;J$1&amp;"("&amp;J2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(K2="",K2=0,K2="-"),"", "; "&amp;K$1&amp;"("&amp;K2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(L2="",L2=0,L2="-"),"", "; "&amp;L$1&amp;"("&amp;L2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(M2="",M2=0,M2="-"),"", "; "&amp;M$1&amp;"("&amp;M2&amp;")("&amp;$C2&amp;")")&amp;
+IF(OR(N2="",N2=0,N2="-"),"", "; "&amp;N$1&amp;"("&amp;N2&amp;")("&amp;$C2&amp;")")</f>
+        <v>Qulub(25000)(belanja); Lintang(25000)(belanja); Yohn(25000)(belanja); Aldo(25000)(belanja); Haqqi(25000)(belanja); Acha(25000)(belanja)</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2">
+        <f>100000/4</f>
+        <v>25000</v>
+      </c>
+      <c r="J2">
+        <f t="shared" ref="J2:N7" si="0">100000/4</f>
+        <v>25000</v>
+      </c>
+      <c r="K2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="L2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="M2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="N2">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>46270</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3">
+        <v>273000</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <f>IF(OR(I3="",I3=0,I3="-"),"",I$1&amp;"("&amp;I3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(J3="",J3=0,J3="-"),"",IF(I3="", "", "; ")&amp;J$1&amp;"("&amp;J3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(K3="",K3=0,K3="-"),"", "; "&amp;K$1&amp;"("&amp;K3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(L3="",L3=0,L3="-"),"", "; "&amp;L$1&amp;"("&amp;L3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(M3="",M3=0,M3="-"),"", "; "&amp;M$1&amp;"("&amp;M3&amp;")("&amp;$C3&amp;")")&amp;
+IF(OR(N3="",N3=0,N3="-"),"", "; "&amp;N$1&amp;"("&amp;N3&amp;")("&amp;$C3&amp;")")</f>
+        <v>Qulub(25000)(belanja); Lintang(25000)(belanja); Yohn(45000)(belanja); Aldo(43000)(belanja); Acha(34200)(belanja)</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I7" si="1">100000/4</f>
+        <v>25000</v>
+      </c>
+      <c r="J3">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="K3">
+        <v>45000</v>
+      </c>
+      <c r="L3">
+        <v>43000</v>
+      </c>
+      <c r="N3">
+        <v>34200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46270</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4">
+        <v>273000</v>
+      </c>
+      <c r="F4" s="2" t="str">
+        <f t="shared" ref="F4" si="2">IF(OR(I4="",I4=0,I4="-"),"",I$1&amp;"("&amp;I4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(J4="",J4=0,J4="-"),"",IF(I4="", "", "; ")&amp;J$1&amp;"("&amp;J4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(K4="",K4=0,K4="-"),"", "; "&amp;K$1&amp;"("&amp;K4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(L4="",L4=0,L4="-"),"", "; "&amp;L$1&amp;"("&amp;L4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(M4="",M4=0,M4="-"),"", "; "&amp;M$1&amp;"("&amp;M4&amp;")("&amp;$C4&amp;")")&amp;
+IF(OR(N4="",N4=0,N4="-"),"", "; "&amp;N$1&amp;"("&amp;N4&amp;")("&amp;$C4&amp;")")</f>
+        <v>Qulub(25000)(belanja); Lintang(25000)(belanja); Acha(34200)(belanja)</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="1"/>
+        <v>25000</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="N4">
+        <v>34200</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>46270</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <f>SUM(I5:N5)</f>
+        <v>84200</v>
+      </c>
+      <c r="F5" s="2" t="str">
+        <f>IF(OR(I5="",I5=0,I5="-"),"",I$1&amp;"("&amp;I5&amp;")("&amp;$C5&amp;")")&amp;
+IF(OR(J5="",J5=0,J5="-"),"",IF(I5="", "", "; ")&amp;J$1&amp;"("&amp;J5&amp;")("&amp;$C5&amp;")")&amp;
+IF(OR(K5="",K5=0,K5="-"),"", "; "&amp;K$1&amp;"("&amp;K5&amp;")("&amp;$C5&amp;")")&amp;
+IF(OR(L5="",L5=0,L5="-"),"", "; "&amp;L$1&amp;"("&amp;L5&amp;")("&amp;$C5&amp;")")&amp;
+IF(OR(M5="",M5=0,M5="-"),"", "; "&amp;M$1&amp;"("&amp;M5&amp;")("&amp;$C5&amp;")")&amp;
+IF(OR(N5="",N5=0,N5="-"),"", "; "&amp;N$1&amp;"("&amp;N5&amp;")("&amp;$C5&amp;")")</f>
+        <v>Qulub(25000)(belanja); Lintang(25000)(belanja); Haqqi(34200)(belanja)</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="1"/>
+        <v>25000</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="M5">
+        <v>34200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>46270</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6">
+        <v>273000</v>
+      </c>
+      <c r="F6" s="2" t="str">
+        <f>IF(OR(I6="",I6=0,I6="-"),"",I$1&amp;"("&amp;I6&amp;")("&amp;$C6&amp;")")&amp;
+IF(OR(J6="",J6=0,J6="-"),"",IF(I6="", "", "; ")&amp;J$1&amp;"("&amp;J6&amp;")("&amp;$C6&amp;")")&amp;
+IF(OR(K6="",K6=0,K6="-"),"", "; "&amp;K$1&amp;"("&amp;K6&amp;")("&amp;$C6&amp;")")&amp;
+IF(OR(L6="",L6=0,L6="-"),"", "; "&amp;L$1&amp;"("&amp;L6&amp;")("&amp;$C6&amp;")")&amp;
+IF(OR(M6="",M6=0,M6="-"),"", "; "&amp;M$1&amp;"("&amp;M6&amp;")("&amp;$C6&amp;")")&amp;
+IF(OR(N6="",N6=0,N6="-"),"", "; "&amp;N$1&amp;"("&amp;N6&amp;")("&amp;$C6&amp;")")</f>
+        <v>Qulub(25000)(belanja); Lintang(25000)(belanja); Aldo(34200)(belanja)</v>
+      </c>
+      <c r="G6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="1"/>
+        <v>25000</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="L6">
+        <v>34200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>46270</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7">
+        <v>273000</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <f t="shared" ref="F7" si="3">IF(OR(I7="",I7=0,I7="-"),"",I$1&amp;"("&amp;I7&amp;")("&amp;$C7&amp;")")&amp;
+IF(OR(J7="",J7=0,J7="-"),"",IF(I7="", "", "; ")&amp;J$1&amp;"("&amp;J7&amp;")("&amp;$C7&amp;")")&amp;
+IF(OR(K7="",K7=0,K7="-"),"", "; "&amp;K$1&amp;"("&amp;K7&amp;")("&amp;$C7&amp;")")&amp;
+IF(OR(L7="",L7=0,L7="-"),"", "; "&amp;L$1&amp;"("&amp;L7&amp;")("&amp;$C7&amp;")")&amp;
+IF(OR(M7="",M7=0,M7="-"),"", "; "&amp;M$1&amp;"("&amp;M7&amp;")("&amp;$C7&amp;")")&amp;
+IF(OR(N7="",N7=0,N7="-"),"", "; "&amp;N$1&amp;"("&amp;N7&amp;")("&amp;$C7&amp;")")</f>
+        <v>Qulub(25000)(belanja); Lintang(25000)(belanja); Yohn(34200)(belanja); Acha(34200)(belanja)</v>
+      </c>
+      <c r="G7" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="1"/>
+        <v>25000</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>25000</v>
+      </c>
+      <c r="K7">
+        <v>34200</v>
+      </c>
+      <c r="N7">
+        <v>34200</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G7">
+      <formula1>"Pending, Selesai"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>